<commit_message>
Update project management Excel sheets with actual Milestone 2 test cases, defects, and sprint backlog
</commit_message>
<xml_diff>
--- a/Unit_Test_Plan_v0.1.xlsx
+++ b/Unit_Test_Plan_v0.1.xlsx
@@ -1,95 +1,53 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://infosystechnologies-my.sharepoint.com/personal/kamaljeet_kaur01_ad_infosys_com1/Documents/Infosys/CC/Events/Oct 2021 - Mar 2022/CC2.0/Internship/Jan-Apr 2022/Artifacts/internship/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B9D4FEA-5A3F-460B-9A40-165575443B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{C3B83BB6-2AB9-4547-8541-9F6969E92BF1}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="UT" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UT" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Actual Result</t>
-  </si>
-  <si>
-    <t>Expected Result</t>
-  </si>
-  <si>
-    <t>Condition to be tested</t>
-  </si>
-  <si>
-    <t>Test Procedure</t>
-  </si>
-  <si>
-    <t>Test Case Name</t>
-  </si>
-  <si>
-    <t>Sl: No:</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color indexed="56"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color indexed="56"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="0"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.39997558519241921"/>
+        <fgColor theme="3" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -122,27 +80,86 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -442,79 +459,205 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF95B16C-182C-4757-B929-A728708A2DB0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="5" width="16.5703125" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" customWidth="1"/>
+    <col width="9.140625" customWidth="1" min="1" max="1"/>
+    <col width="14.28515625" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16.5703125" customWidth="1" min="4" max="5"/>
+    <col width="15.85546875" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="31.5" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" ht="31.5" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Sl: No:</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Test Case Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Test Procedure</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Condition to be tested</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>TC01 - Clean Java Code</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Run Code Analysis on clean Java snippet</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Ensure PMD and SpotBugs return 0 false positives</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>No findings</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>TC02 - Java Multiple Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Run Security Analysis on Java snippet with Runtime.exec()</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Ensure FindSecBugs catches COMMAND_INJECTION</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>High Severity Command Injection detected</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>TC03 - Python Injection Snippet</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Run Security Analysis on Python with eval() and exec()</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Ensure Bandit catches B307 and B102</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>High Severity Code Injection detected</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>TC04 - Multi-Agent Orchestration</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Submit snippet to LangGraph orchestrator endpoint</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Ensure Code Analysis and Security Analysis run in parallel</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Merged findings array returned</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>TC05 - Frontend API Calls</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Click export markdown and view chat history in UI</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Ensure UI correctly proxies to backend without IPv6 refusal</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Data loads successfully</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>